<commit_message>
feat: connect query expansion to hybrid retrieval
</commit_message>
<xml_diff>
--- a/docs/exam_proof/回归测试结果_20260918_修订版.xlsx
+++ b/docs/exam_proof/回归测试结果_20260918_修订版.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 16:49:16</t>
+          <t>2026-10-03 18:07:09</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>a01f9cd</t>
+          <t>c4be1d9</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0.47</v>
+        <v>0.35</v>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>D:\社团考题第八\data\corpus\clauses.jsonl</t>
+          <t>D:\社团考题第八\knowledge\pure_kb\data\clauses.jsonl</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.77</v>
+        <v>0.79</v>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
     </row>
@@ -975,7 +975,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>D:\社团考题第八\vector_kb\bm25_index.pkl</t>
+          <t>D:\社团考题第八\knowledge\pure_kb\index\bm25_index.pkl</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.19</v>
+        <v>1.17</v>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>D:\社团考题第八\vector_kb\knowledge.db</t>
+          <t>D:\社团考题第八\knowledge\pure_kb\index\knowledge.db</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>3.44</v>
+        <v>3.05</v>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
     </row>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.29</v>
+        <v>0.31</v>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
     </row>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
     </row>
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>98.59999999999999</v>
+        <v>88.68000000000001</v>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
     </row>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>62.27</v>
+        <v>39.12</v>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
     </row>
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>365.85</v>
+        <v>367.7</v>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
     </row>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>1</v>
+        <v>1.21</v>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
     </row>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>55.37</v>
+        <v>68.14</v>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
     </row>
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>60.82</v>
+        <v>95.76000000000001</v>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
     </row>
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>60.07</v>
+        <v>39.61</v>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
     </row>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>49.53</v>
+        <v>59.07</v>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
     </row>
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>39.44</v>
+        <v>66.75</v>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
     </row>
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
     </row>
@@ -2391,7 +2391,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="51" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>D:\社团考题第八\data\corpus\clauses.jsonl</t>
+          <t>D:\社团考题第八\knowledge\pure_kb\data\clauses.jsonl</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>D:\社团考题第八\vector_kb\bm25_index.pkl</t>
+          <t>D:\社团考题第八\knowledge\pure_kb\index\bm25_index.pkl</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>D:\社团考题第八\vector_kb\knowledge.db</t>
+          <t>D:\社团考题第八\knowledge\pure_kb\index\knowledge.db</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: filter hybrid retrieval by domains
</commit_message>
<xml_diff>
--- a/docs/exam_proof/回归测试结果_20260918_修订版.xlsx
+++ b/docs/exam_proof/回归测试结果_20260918_修订版.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 18:07:09</t>
+          <t>2026-10-03 18:35:47</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>c4be1d9</t>
+          <t>dfab20e</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0.35</v>
+        <v>1.31</v>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
     </row>
@@ -748,7 +748,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
     </row>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
     </row>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.79</v>
+        <v>1.07</v>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
     </row>
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.17</v>
+        <v>1.65</v>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>3.05</v>
+        <v>4.26</v>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
     </row>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
     </row>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
     </row>
@@ -1158,7 +1158,7 @@
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
     </row>
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>88.68000000000001</v>
+        <v>90.87</v>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
     </row>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>39.12</v>
+        <v>73.03</v>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
     </row>
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>367.7</v>
+        <v>362.79</v>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
     </row>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>1.21</v>
+        <v>1.67</v>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
     </row>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>68.14</v>
+        <v>58.04</v>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
     </row>
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>95.76000000000001</v>
+        <v>61.52</v>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
     </row>
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>39.61</v>
+        <v>62.23</v>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
     </row>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>59.07</v>
+        <v>79.44</v>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
     </row>
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>66.75</v>
+        <v>58.82</v>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
refactor: extract chunk filter from knowledge adapter
</commit_message>
<xml_diff>
--- a/docs/exam_proof/回归测试结果_20260918_修订版.xlsx
+++ b/docs/exam_proof/回归测试结果_20260918_修订版.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 18:35:47</t>
+          <t>2026-10-03 19:07:30</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>dfab20e</t>
+          <t>569f693</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.31</v>
+        <v>0.37</v>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
     </row>
@@ -748,7 +748,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
     </row>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
     </row>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.07</v>
+        <v>0.83</v>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
     </row>
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.65</v>
+        <v>1.17</v>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>4.26</v>
+        <v>2.86</v>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
     </row>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
     </row>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
     </row>
@@ -1158,7 +1158,7 @@
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
     </row>
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>90.87</v>
+        <v>71.42</v>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
     </row>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>73.03</v>
+        <v>58.73</v>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
     </row>
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>362.79</v>
+        <v>361.93</v>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
     </row>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>1.67</v>
+        <v>1.41</v>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
     </row>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>58.04</v>
+        <v>63.76</v>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>9.3.1-表3(0.0328)；9.3.2-表4(0.0323)；10.2.1-表6(0.0315)；10.2.3.1(0.0315)；5.6.1(0.0154)</t>
+          <t>9.3.1-表3(0.0328)；9.3.2-表4(0.0323)；10.2.3.1(0.0315)；10.2.1-表6(0.0315)；5.6.1(0.0154)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>61.52</v>
+        <v>97.18000000000001</v>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
     </row>
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>62.23</v>
+        <v>55.45</v>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
     </row>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>6.5.2(0.0164)；10.2.1-表7(0.0164)；6.2.3(0.0161)；6.5.1(0.0159)；4.2.1(0.0156)</t>
+          <t>10.2.1-表7(0.0164)；6.5.2(0.0164)；6.2.3(0.0161)；6.5.1(0.0159)；4.2.1(0.0156)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>79.44</v>
+        <v>63.61</v>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
     </row>
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>58.82</v>
+        <v>46.7</v>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
     </row>
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
     </row>
@@ -1679,7 +1679,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="53" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
+          <t>10.2.3.1</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
           <t>10.2.1-表6</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>10.2.3.1</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -2103,12 +2103,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>10.2.1-表7</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>6.5.2</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>10.2.1-表7</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: support hierarchical clause citations
</commit_message>
<xml_diff>
--- a/docs/exam_proof/回归测试结果_20260918_修订版.xlsx
+++ b/docs/exam_proof/回归测试结果_20260918_修订版.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 19:07:30</t>
+          <t>2026-10-03 19:53:24</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>569f693</t>
+          <t>35608e9</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0.37</v>
+        <v>0.79</v>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
     </row>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
     </row>
@@ -830,7 +830,7 @@
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.06</v>
+        <v>0.03</v>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
     </row>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.83</v>
+        <v>5.32</v>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
     </row>
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.17</v>
+        <v>11.49</v>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>2.86</v>
+        <v>5.1</v>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
     </row>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
     </row>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
     </row>
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>71.42</v>
+        <v>95.27</v>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
     </row>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>58.73</v>
+        <v>98.43000000000001</v>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
     </row>
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>361.93</v>
+        <v>332.3</v>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
     </row>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>1.41</v>
+        <v>1.58</v>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
     </row>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>63.76</v>
+        <v>82.03</v>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
     </row>
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>97.18000000000001</v>
+        <v>59.09</v>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
     </row>
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>55.45</v>
+        <v>62.68</v>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
     </row>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>63.61</v>
+        <v>75.86</v>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
     </row>
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46.7</v>
+        <v>65.48</v>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
     </row>
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
docs: mark legacy retrieval modules deprecated
</commit_message>
<xml_diff>
--- a/docs/exam_proof/回归测试结果_20260918_修订版.xlsx
+++ b/docs/exam_proof/回归测试结果_20260918_修订版.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 19:53:24</t>
+          <t>2026-10-03 20:29:11</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>35608e9</t>
+          <t>bf78a6d</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0.79</v>
+        <v>1.88</v>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
     </row>
@@ -748,7 +748,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
     </row>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
     </row>
@@ -830,7 +830,7 @@
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
     </row>
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
     </row>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>5.32</v>
+        <v>1.67</v>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
     </row>
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>11.49</v>
+        <v>2.04</v>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>5.1</v>
+        <v>4.36</v>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
     </row>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.33</v>
+        <v>0.53</v>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
     </row>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0.25</v>
+        <v>0.53</v>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
     </row>
@@ -1158,7 +1158,7 @@
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>0.21</v>
+        <v>0.29</v>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
     </row>
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>95.27</v>
+        <v>2870.21</v>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
     </row>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>98.43000000000001</v>
+        <v>84.03</v>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
     </row>
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>332.3</v>
+        <v>404.39</v>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
     </row>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>1.58</v>
+        <v>1.34</v>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
     </row>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>82.03</v>
+        <v>79.63</v>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
     </row>
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>59.09</v>
+        <v>61.24</v>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
     </row>
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>62.68</v>
+        <v>62.65</v>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
     </row>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>75.86</v>
+        <v>63.08</v>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
     </row>
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>65.48</v>
+        <v>40.6</v>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
     </row>

</xml_diff>